<commit_message>
chore(ro-crate): sync from Google Sheets
</commit_message>
<xml_diff>
--- a/ro-crate/ro-crate-metadata.xlsx
+++ b/ro-crate/ro-crate-metadata.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="9">
   <si>
     <t>Name</t>
   </si>
@@ -33,6 +33,9 @@
   </si>
   <si>
     <t>hasPart</t>
+  </si>
+  <si>
+    <t/>
   </si>
   <si>
     <t>name</t>
@@ -443,9 +446,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>6</v>
+      </c>
+      <c r="B4" t="s">
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -465,7 +471,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B1" t="s">
         <v>2</v>

</xml_diff>

<commit_message>
updated readme, changed some behaviour deleting before updating
</commit_message>
<xml_diff>
--- a/ro-crate/ro-crate-metadata.xlsx
+++ b/ro-crate/ro-crate-metadata.xlsx
@@ -12,14 +12,13 @@
     <sheet sheetId="6" name="@type=ldac_DataReuseLicense" state="visible" r:id="rId9"/>
     <sheet sheetId="7" name="@type=SoftwareApplication" state="visible" r:id="rId10"/>
     <sheet sheetId="8" name="@type=RepositoryCollection" state="visible" r:id="rId11"/>
-    <sheet sheetId="9" name="@type=DigitalFormat" state="visible" r:id="rId12"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="640" uniqueCount="307">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="623" uniqueCount="299">
   <si>
     <t>Name</t>
   </si>
@@ -60,7 +59,7 @@
     <t>datePublished</t>
   </si>
   <si>
-    <t>Sat Apr 11 2026 00:00:00 GMT+0000 (Coordinated Universal Time)</t>
+    <t>Sat Apr 11 2026 10:00:00 GMT+1000 (Australian Eastern Standard Time)</t>
   </si>
   <si>
     <t>inLanguage</t>
@@ -99,7 +98,7 @@
     <t>hasPart</t>
   </si>
   <si>
-    <t>["additional-ro-crate-metadata.xlsx", "images"]</t>
+    <t>"images"</t>
   </si>
   <si>
     <t>ldac</t>
@@ -114,229 +113,214 @@
     <t>arcp://name,custom/terms#</t>
   </si>
   <si>
-    <t>contentSize</t>
-  </si>
-  <si>
-    <t>dateModified</t>
+    <t>test_file.jpg</t>
+  </si>
+  <si>
+    <t>File</t>
+  </si>
+  <si>
+    <t>https://orcid.org/0000-0002-1428-2649</t>
+  </si>
+  <si>
+    <t>Person</t>
+  </si>
+  <si>
+    <t>Chao Sun</t>
+  </si>
+  <si>
+    <t>https://orcid.org/0009-0008-4603-9521</t>
+  </si>
+  <si>
+    <t>Jasper Chong</t>
+  </si>
+  <si>
+    <t>#JohnHatton</t>
+  </si>
+  <si>
+    <t>John Hatton</t>
+  </si>
+  <si>
+    <t>https://orcid.org/0000-0002-3616-6235</t>
+  </si>
+  <si>
+    <t>Marius Mather</t>
+  </si>
+  <si>
+    <t>https://orcid.org/0000-0003-1923-9153</t>
+  </si>
+  <si>
+    <t>Martin Schweinberger</t>
+  </si>
+  <si>
+    <t>https://orcid.org/0000-0002-4438-2755</t>
+  </si>
+  <si>
+    <t>Moises Sacal Bonequi</t>
+  </si>
+  <si>
+    <t>https://orcid.org/0000-0001-8797-1018</t>
+  </si>
+  <si>
+    <t>Nick Thieberger</t>
+  </si>
+  <si>
+    <t>https://orcid.org/0000-0003-2933-6627</t>
+  </si>
+  <si>
+    <t>Robert Fleet</t>
+  </si>
+  <si>
+    <t>https://orcid.org/0000-0002-1824-2361</t>
+  </si>
+  <si>
+    <t>Sam Hames</t>
+  </si>
+  <si>
+    <t>#SonyJufri</t>
+  </si>
+  <si>
+    <t>Sony Jufri</t>
+  </si>
+  <si>
+    <t>https://orcid.org/0000-0003-4904-2941</t>
+  </si>
+  <si>
+    <t>Wolfgang Barth</t>
+  </si>
+  <si>
+    <t>https://orcid.org/0000-0002-2118-3147</t>
+  </si>
+  <si>
+    <t>River Tae Smith</t>
+  </si>
+  <si>
+    <t>https://orcid.org/0009-0006-2241-3377</t>
+  </si>
+  <si>
+    <t>Rosanna Smith</t>
+  </si>
+  <si>
+    <t>https://orcid.org/0000-0003-3237-9943</t>
+  </si>
+  <si>
+    <t>Simon Musgrave</t>
+  </si>
+  <si>
+    <t>https://github.com/Language-Research-Technology</t>
+  </si>
+  <si>
+    <t>Organization</t>
+  </si>
+  <si>
+    <t>Language Data Commons of Australia</t>
+  </si>
+  <si>
+    <t>https://ror.org/00rqy9422</t>
+  </si>
+  <si>
+    <t>The University of Queensland</t>
+  </si>
+  <si>
+    <t>https://ror.org/019wvm592</t>
+  </si>
+  <si>
+    <t>Australian National University</t>
+  </si>
+  <si>
+    <t>https://ror.org/01ej9dk98</t>
+  </si>
+  <si>
+    <t>The University of Melbourne</t>
+  </si>
+  <si>
+    <t>https://ror.org/0384j8v12</t>
+  </si>
+  <si>
+    <t>The University of Sydney</t>
+  </si>
+  <si>
+    <t>https://ror.org/03pnv4752</t>
+  </si>
+  <si>
+    <t>Queensland University of Technology</t>
+  </si>
+  <si>
+    <t>https://github.com/Sydney-Informatics-Hub</t>
+  </si>
+  <si>
+    <t>Sydney Informatics Hub</t>
+  </si>
+  <si>
+    <t>https://github.com/QUT-Digital-Observatory</t>
+  </si>
+  <si>
+    <t>Digital Observatory</t>
+  </si>
+  <si>
+    <t>https://github.com/SLCLADAL/ladal</t>
+  </si>
+  <si>
+    <t>Language Technology and Data Analysis Laboratory</t>
+  </si>
+  <si>
+    <t>https://hass.uq.edu.au/centre-digital-cultures-societies</t>
+  </si>
+  <si>
+    <t>Centre for Digital Cultures &amp; Societies</t>
+  </si>
+  <si>
+    <t>ldac:allowTextIndex</t>
+  </si>
+  <si>
+    <t>isPartOf</t>
+  </si>
+  <si>
+    <t>https://creativecommons.org/licenses/by/4.0/</t>
+  </si>
+  <si>
+    <t>ldac:DataReuseLicense</t>
+  </si>
+  <si>
+    <t>Attribution 4.0 International (CC BY 4.0)</t>
+  </si>
+  <si>
+    <t>You are free to: Share — copy and redistribute the material in any medium or format. Adapt — remix, transform, and build upon the material for any purpose, even commercially. This license is acceptable for Free Cultural Works. The licensor cannot revoke these freedoms as long as you follow the license terms.</t>
+  </si>
+  <si>
+    <t>"./"</t>
+  </si>
+  <si>
+    <t>conformsTo</t>
+  </si>
+  <si>
+    <t>pcdm:memberOf</t>
+  </si>
+  <si>
+    <t>programmingLanguage</t>
+  </si>
+  <si>
+    <t>url</t>
+  </si>
+  <si>
+    <t>custom:dataFormat</t>
+  </si>
+  <si>
+    <t>custom:codeURL</t>
+  </si>
+  <si>
+    <t>custom:guideURL</t>
+  </si>
+  <si>
+    <t>creditText</t>
+  </si>
+  <si>
+    <t>custom:additionalNotes</t>
+  </si>
+  <si>
+    <t>input</t>
   </si>
   <si>
     <t>encodingFormat</t>
-  </si>
-  <si>
-    <t>test_file.jpg</t>
-  </si>
-  <si>
-    <t>File</t>
-  </si>
-  <si>
-    <t>additional-ro-crate-metadata.xlsx</t>
-  </si>
-  <si>
-    <t>2026-08-19T02:36:29Z</t>
-  </si>
-  <si>
-    <t>["https://www.nationalarchives.gov.uk/PRONOM/fmt/214", application/vnd.openxmlformats-officedocument.spreadsheetml.sheet]</t>
-  </si>
-  <si>
-    <t>https://orcid.org/0000-0002-1428-2649</t>
-  </si>
-  <si>
-    <t>Person</t>
-  </si>
-  <si>
-    <t>Chao Sun</t>
-  </si>
-  <si>
-    <t>https://orcid.org/0009-0008-4603-9521</t>
-  </si>
-  <si>
-    <t>Jasper Chong</t>
-  </si>
-  <si>
-    <t>#JohnHatton</t>
-  </si>
-  <si>
-    <t>John Hatton</t>
-  </si>
-  <si>
-    <t>https://orcid.org/0000-0002-3616-6235</t>
-  </si>
-  <si>
-    <t>Marius Mather</t>
-  </si>
-  <si>
-    <t>https://orcid.org/0000-0003-1923-9153</t>
-  </si>
-  <si>
-    <t>Martin Schweinberger</t>
-  </si>
-  <si>
-    <t>https://orcid.org/0000-0002-4438-2755</t>
-  </si>
-  <si>
-    <t>Moises Sacal Bonequi</t>
-  </si>
-  <si>
-    <t>https://orcid.org/0000-0001-8797-1018</t>
-  </si>
-  <si>
-    <t>Nick Thieberger</t>
-  </si>
-  <si>
-    <t>https://orcid.org/0000-0003-2933-6627</t>
-  </si>
-  <si>
-    <t>Robert Fleet</t>
-  </si>
-  <si>
-    <t>https://orcid.org/0000-0002-1824-2361</t>
-  </si>
-  <si>
-    <t>Sam Hames</t>
-  </si>
-  <si>
-    <t>#SonyJufri</t>
-  </si>
-  <si>
-    <t>Sony Jufri</t>
-  </si>
-  <si>
-    <t>https://orcid.org/0000-0003-4904-2941</t>
-  </si>
-  <si>
-    <t>Wolfgang Barth</t>
-  </si>
-  <si>
-    <t>https://orcid.org/0000-0002-2118-3147</t>
-  </si>
-  <si>
-    <t>River Tae Smith</t>
-  </si>
-  <si>
-    <t>https://orcid.org/0009-0006-2241-3377</t>
-  </si>
-  <si>
-    <t>Rosanna Smith</t>
-  </si>
-  <si>
-    <t>https://orcid.org/0000-0003-3237-9943</t>
-  </si>
-  <si>
-    <t>Simon Musgrave</t>
-  </si>
-  <si>
-    <t>https://github.com/Language-Research-Technology</t>
-  </si>
-  <si>
-    <t>Organization</t>
-  </si>
-  <si>
-    <t>Language Data Commons of Australia</t>
-  </si>
-  <si>
-    <t>https://ror.org/00rqy9422</t>
-  </si>
-  <si>
-    <t>The University of Queensland</t>
-  </si>
-  <si>
-    <t>https://ror.org/019wvm592</t>
-  </si>
-  <si>
-    <t>Australian National University</t>
-  </si>
-  <si>
-    <t>https://ror.org/01ej9dk98</t>
-  </si>
-  <si>
-    <t>The University of Melbourne</t>
-  </si>
-  <si>
-    <t>https://ror.org/0384j8v12</t>
-  </si>
-  <si>
-    <t>The University of Sydney</t>
-  </si>
-  <si>
-    <t>https://ror.org/03pnv4752</t>
-  </si>
-  <si>
-    <t>Queensland University of Technology</t>
-  </si>
-  <si>
-    <t>https://github.com/Sydney-Informatics-Hub</t>
-  </si>
-  <si>
-    <t>Sydney Informatics Hub</t>
-  </si>
-  <si>
-    <t>https://github.com/QUT-Digital-Observatory</t>
-  </si>
-  <si>
-    <t>Digital Observatory</t>
-  </si>
-  <si>
-    <t>https://github.com/SLCLADAL/ladal</t>
-  </si>
-  <si>
-    <t>Language Technology and Data Analysis Laboratory</t>
-  </si>
-  <si>
-    <t>https://hass.uq.edu.au/centre-digital-cultures-societies</t>
-  </si>
-  <si>
-    <t>Centre for Digital Cultures &amp; Societies</t>
-  </si>
-  <si>
-    <t>ldac:allowTextIndex</t>
-  </si>
-  <si>
-    <t>isPartOf</t>
-  </si>
-  <si>
-    <t>https://creativecommons.org/licenses/by/4.0/</t>
-  </si>
-  <si>
-    <t>ldac:DataReuseLicense</t>
-  </si>
-  <si>
-    <t>Attribution 4.0 International (CC BY 4.0)</t>
-  </si>
-  <si>
-    <t>You are free to: Share — copy and redistribute the material in any medium or format. Adapt — remix, transform, and build upon the material for any purpose, even commercially. This license is acceptable for Free Cultural Works. The licensor cannot revoke these freedoms as long as you follow the license terms.</t>
-  </si>
-  <si>
-    <t>"./"</t>
-  </si>
-  <si>
-    <t>conformsTo</t>
-  </si>
-  <si>
-    <t>pcdm:memberOf</t>
-  </si>
-  <si>
-    <t>programmingLanguage</t>
-  </si>
-  <si>
-    <t>url</t>
-  </si>
-  <si>
-    <t>custom:dataFormat</t>
-  </si>
-  <si>
-    <t>custom:codeURL</t>
-  </si>
-  <si>
-    <t>custom:guideURL</t>
-  </si>
-  <si>
-    <t>creditText</t>
-  </si>
-  <si>
-    <t>custom:additionalNotes</t>
-  </si>
-  <si>
-    <t>input</t>
   </si>
   <si>
     <t>arcp://name,AnonymisingELANFiles</t>
@@ -859,7 +843,7 @@
     <t>Farms to freeways notebook</t>
   </si>
   <si>
-    <t>Sun Jul 07 2024 00:00:00 GMT+0000 (Coordinated Universal Time)</t>
+    <t>Sun Jul 07 2024 10:00:00 GMT+1000 (Australian Eastern Standard Time)</t>
   </si>
   <si>
     <t>"Mel Mistica"</t>
@@ -932,15 +916,6 @@
   </si>
   <si>
     <t>Australian Twittersphere (AuTS) aggregated data - Collection</t>
-  </si>
-  <si>
-    <t>https://www.nationalarchives.gov.uk/PRONOM/fmt/214</t>
-  </si>
-  <si>
-    <t>DigitalFormat</t>
-  </si>
-  <si>
-    <t>Microsoft Excel for Windows</t>
   </si>
 </sst>
 </file>
@@ -1483,64 +1458,26 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="7" width="20" customWidth="1"/>
+    <col min="1" max="2" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>2</v>
       </c>
       <c r="B1" t="s">
         <v>4</v>
       </c>
-      <c r="C1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E1" t="s">
-        <v>31</v>
-      </c>
-      <c r="F1" t="s">
-        <v>32</v>
-      </c>
-      <c r="G1" t="s">
-        <v>33</v>
-      </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>36</v>
-      </c>
-      <c r="B3" t="s">
-        <v>35</v>
-      </c>
-      <c r="C3" t="s">
-        <v>36</v>
-      </c>
-      <c r="D3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E3">
-        <v>16253</v>
-      </c>
-      <c r="F3" t="s">
-        <v>37</v>
-      </c>
-      <c r="G3" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>
@@ -1570,156 +1507,156 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="B2" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="C2" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="B3" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="C3" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="B4" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="C4" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="B5" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="C5" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="B6" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="C6" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="B7" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="C7" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="B8" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="C8" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="B9" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="C9" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="B10" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="C10" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="B11" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="C11" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="B12" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="C12" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="B13" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="C13" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="B14" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="C14" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="B15" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="C15" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
     </row>
   </sheetData>
@@ -1749,112 +1686,112 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="B2" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="C2" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="B3" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="C3" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="B4" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="C4" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="B5" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="C5" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="B6" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="C6" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="B7" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="C7" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="B8" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="C8" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="B9" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="C9" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="B10" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="C10" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="B11" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="C11" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
     </row>
   </sheetData>
@@ -1885,30 +1822,30 @@
         <v>8</v>
       </c>
       <c r="E1" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="F1" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="B2" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="C2" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="D2" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="E2" t="b">
         <v>1</v>
       </c>
       <c r="F2" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
     </row>
   </sheetData>
@@ -1933,10 +1870,10 @@
         <v>4</v>
       </c>
       <c r="C1" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="D1" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="E1" t="s">
         <v>6</v>
@@ -1951,1494 +1888,1494 @@
         <v>17</v>
       </c>
       <c r="I1" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="J1" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="K1" t="s">
         <v>8</v>
       </c>
       <c r="L1" t="s">
+        <v>94</v>
+      </c>
+      <c r="M1" t="s">
+        <v>95</v>
+      </c>
+      <c r="N1" t="s">
+        <v>96</v>
+      </c>
+      <c r="O1" t="s">
+        <v>97</v>
+      </c>
+      <c r="P1" t="s">
+        <v>98</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>99</v>
+      </c>
+      <c r="R1" t="s">
         <v>100</v>
-      </c>
-      <c r="M1" t="s">
-        <v>101</v>
-      </c>
-      <c r="N1" t="s">
-        <v>102</v>
-      </c>
-      <c r="O1" t="s">
-        <v>103</v>
-      </c>
-      <c r="P1" t="s">
-        <v>104</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>105</v>
-      </c>
-      <c r="R1" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="B2" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="C2" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="D2" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="E2" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="F2" t="s">
         <v>13</v>
       </c>
       <c r="G2" t="s">
+        <v>105</v>
+      </c>
+      <c r="H2" t="s">
+        <v>106</v>
+      </c>
+      <c r="I2" t="s">
+        <v>107</v>
+      </c>
+      <c r="J2" t="s">
+        <v>108</v>
+      </c>
+      <c r="K2" t="s">
+        <v>109</v>
+      </c>
+      <c r="L2" t="s">
         <v>110</v>
       </c>
-      <c r="H2" t="s">
-        <v>111</v>
-      </c>
-      <c r="I2" t="s">
-        <v>112</v>
-      </c>
-      <c r="J2" t="s">
-        <v>113</v>
-      </c>
-      <c r="K2" t="s">
-        <v>114</v>
-      </c>
-      <c r="L2" t="s">
-        <v>115</v>
-      </c>
       <c r="M2" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="B3" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="C3" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="D3" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="E3" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="F3" t="s">
         <v>13</v>
       </c>
       <c r="G3" t="s">
+        <v>113</v>
+      </c>
+      <c r="H3" t="s">
+        <v>114</v>
+      </c>
+      <c r="I3" t="s">
+        <v>115</v>
+      </c>
+      <c r="J3" t="s">
+        <v>116</v>
+      </c>
+      <c r="K3" t="s">
+        <v>117</v>
+      </c>
+      <c r="L3" t="s">
         <v>118</v>
       </c>
-      <c r="H3" t="s">
+      <c r="M3" t="s">
         <v>119</v>
-      </c>
-      <c r="I3" t="s">
-        <v>120</v>
-      </c>
-      <c r="J3" t="s">
-        <v>121</v>
-      </c>
-      <c r="K3" t="s">
-        <v>122</v>
-      </c>
-      <c r="L3" t="s">
-        <v>123</v>
-      </c>
-      <c r="M3" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="B4" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="C4" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="D4" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="E4" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="F4" t="s">
         <v>13</v>
       </c>
       <c r="G4" t="s">
+        <v>113</v>
+      </c>
+      <c r="H4" t="s">
+        <v>114</v>
+      </c>
+      <c r="I4" t="s">
+        <v>122</v>
+      </c>
+      <c r="J4" t="s">
+        <v>123</v>
+      </c>
+      <c r="K4" t="s">
+        <v>124</v>
+      </c>
+      <c r="L4" t="s">
         <v>118</v>
       </c>
-      <c r="H4" t="s">
-        <v>119</v>
-      </c>
-      <c r="I4" t="s">
-        <v>127</v>
-      </c>
-      <c r="J4" t="s">
-        <v>128</v>
-      </c>
-      <c r="K4" t="s">
-        <v>129</v>
-      </c>
-      <c r="L4" t="s">
-        <v>123</v>
-      </c>
       <c r="M4" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="B5" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="C5" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="D5" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="E5" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="F5" t="s">
         <v>13</v>
       </c>
       <c r="G5" t="s">
+        <v>113</v>
+      </c>
+      <c r="H5" t="s">
+        <v>114</v>
+      </c>
+      <c r="I5" t="s">
+        <v>115</v>
+      </c>
+      <c r="J5" t="s">
+        <v>116</v>
+      </c>
+      <c r="K5" t="s">
+        <v>128</v>
+      </c>
+      <c r="L5" t="s">
         <v>118</v>
       </c>
-      <c r="H5" t="s">
-        <v>119</v>
-      </c>
-      <c r="I5" t="s">
-        <v>120</v>
-      </c>
-      <c r="J5" t="s">
-        <v>121</v>
-      </c>
-      <c r="K5" t="s">
-        <v>133</v>
-      </c>
-      <c r="L5" t="s">
-        <v>123</v>
-      </c>
       <c r="M5" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="B6" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="C6" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="D6" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="E6" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="F6" t="s">
         <v>13</v>
       </c>
       <c r="G6" t="s">
+        <v>132</v>
+      </c>
+      <c r="H6" t="s">
+        <v>133</v>
+      </c>
+      <c r="I6" t="s">
+        <v>107</v>
+      </c>
+      <c r="J6" t="s">
+        <v>134</v>
+      </c>
+      <c r="K6" t="s">
+        <v>135</v>
+      </c>
+      <c r="L6" t="s">
+        <v>136</v>
+      </c>
+      <c r="M6" t="s">
+        <v>134</v>
+      </c>
+      <c r="N6" t="s">
         <v>137</v>
       </c>
-      <c r="H6" t="s">
+      <c r="O6" t="s">
         <v>138</v>
-      </c>
-      <c r="I6" t="s">
-        <v>112</v>
-      </c>
-      <c r="J6" t="s">
-        <v>139</v>
-      </c>
-      <c r="K6" t="s">
-        <v>140</v>
-      </c>
-      <c r="L6" t="s">
-        <v>141</v>
-      </c>
-      <c r="M6" t="s">
-        <v>139</v>
-      </c>
-      <c r="N6" t="s">
-        <v>142</v>
-      </c>
-      <c r="O6" t="s">
-        <v>143</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="B7" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="C7" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="D7" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="E7" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="F7" t="s">
         <v>13</v>
       </c>
       <c r="G7" t="s">
+        <v>141</v>
+      </c>
+      <c r="H7" t="s">
+        <v>142</v>
+      </c>
+      <c r="I7" t="s">
+        <v>122</v>
+      </c>
+      <c r="J7" t="s">
+        <v>143</v>
+      </c>
+      <c r="K7" t="s">
+        <v>144</v>
+      </c>
+      <c r="L7" t="s">
+        <v>145</v>
+      </c>
+      <c r="M7" t="s">
+        <v>143</v>
+      </c>
+      <c r="N7" t="s">
         <v>146</v>
-      </c>
-      <c r="H7" t="s">
-        <v>147</v>
-      </c>
-      <c r="I7" t="s">
-        <v>127</v>
-      </c>
-      <c r="J7" t="s">
-        <v>148</v>
-      </c>
-      <c r="K7" t="s">
-        <v>149</v>
-      </c>
-      <c r="L7" t="s">
-        <v>150</v>
-      </c>
-      <c r="M7" t="s">
-        <v>148</v>
-      </c>
-      <c r="N7" t="s">
-        <v>151</v>
       </c>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="B8" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="C8" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="D8" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="E8" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="F8" t="s">
         <v>13</v>
       </c>
       <c r="G8" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="I8" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="J8" t="s">
+        <v>149</v>
+      </c>
+      <c r="K8" t="s">
+        <v>150</v>
+      </c>
+      <c r="L8" t="s">
+        <v>151</v>
+      </c>
+      <c r="M8" t="s">
+        <v>149</v>
+      </c>
+      <c r="N8" t="s">
+        <v>152</v>
+      </c>
+      <c r="O8" t="s">
+        <v>153</v>
+      </c>
+      <c r="P8" t="s">
         <v>154</v>
-      </c>
-      <c r="K8" t="s">
-        <v>155</v>
-      </c>
-      <c r="L8" t="s">
-        <v>156</v>
-      </c>
-      <c r="M8" t="s">
-        <v>154</v>
-      </c>
-      <c r="N8" t="s">
-        <v>157</v>
-      </c>
-      <c r="O8" t="s">
-        <v>158</v>
-      </c>
-      <c r="P8" t="s">
-        <v>159</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="B9" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="C9" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="D9" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="E9" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="F9" t="s">
         <v>13</v>
       </c>
       <c r="G9" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="H9" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="I9" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="J9" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="K9" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="L9" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="M9" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="N9" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="O9" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
       <c r="B10" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="C10" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="D10" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="E10" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="F10" t="s">
         <v>13</v>
       </c>
       <c r="G10" t="s">
+        <v>105</v>
+      </c>
+      <c r="H10" t="s">
+        <v>106</v>
+      </c>
+      <c r="I10" t="s">
+        <v>164</v>
+      </c>
+      <c r="J10" t="s">
+        <v>165</v>
+      </c>
+      <c r="K10" t="s">
+        <v>166</v>
+      </c>
+      <c r="L10" t="s">
         <v>110</v>
       </c>
-      <c r="H10" t="s">
-        <v>111</v>
-      </c>
-      <c r="I10" t="s">
-        <v>169</v>
-      </c>
-      <c r="J10" t="s">
-        <v>170</v>
-      </c>
-      <c r="K10" t="s">
-        <v>171</v>
-      </c>
-      <c r="L10" t="s">
-        <v>115</v>
-      </c>
       <c r="M10" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="B11" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="C11" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="D11" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="E11" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="F11" t="s">
         <v>13</v>
       </c>
       <c r="G11" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="H11" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="I11" t="s">
+        <v>164</v>
+      </c>
+      <c r="J11" t="s">
+        <v>165</v>
+      </c>
+      <c r="K11" t="s">
         <v>169</v>
       </c>
-      <c r="J11" t="s">
+      <c r="L11" t="s">
         <v>170</v>
       </c>
-      <c r="K11" t="s">
-        <v>174</v>
-      </c>
-      <c r="L11" t="s">
-        <v>175</v>
-      </c>
       <c r="M11" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="B12" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="C12" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="D12" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="E12" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="F12" t="s">
         <v>13</v>
       </c>
       <c r="G12" t="s">
+        <v>105</v>
+      </c>
+      <c r="H12" t="s">
+        <v>106</v>
+      </c>
+      <c r="I12" t="s">
+        <v>122</v>
+      </c>
+      <c r="J12" t="s">
+        <v>173</v>
+      </c>
+      <c r="K12" t="s">
+        <v>174</v>
+      </c>
+      <c r="L12" t="s">
         <v>110</v>
       </c>
-      <c r="H12" t="s">
-        <v>111</v>
-      </c>
-      <c r="I12" t="s">
-        <v>127</v>
-      </c>
-      <c r="J12" t="s">
-        <v>178</v>
-      </c>
-      <c r="K12" t="s">
-        <v>179</v>
-      </c>
-      <c r="L12" t="s">
-        <v>115</v>
-      </c>
       <c r="M12" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="B13" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="C13" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="D13" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="E13" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="F13" t="s">
         <v>13</v>
       </c>
       <c r="G13" t="s">
+        <v>105</v>
+      </c>
+      <c r="H13" t="s">
+        <v>106</v>
+      </c>
+      <c r="I13" t="s">
+        <v>122</v>
+      </c>
+      <c r="J13" t="s">
+        <v>177</v>
+      </c>
+      <c r="K13" t="s">
+        <v>178</v>
+      </c>
+      <c r="L13" t="s">
         <v>110</v>
       </c>
-      <c r="H13" t="s">
-        <v>111</v>
-      </c>
-      <c r="I13" t="s">
-        <v>127</v>
-      </c>
-      <c r="J13" t="s">
-        <v>182</v>
-      </c>
-      <c r="K13" t="s">
-        <v>183</v>
-      </c>
-      <c r="L13" t="s">
-        <v>115</v>
-      </c>
       <c r="M13" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="B14" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="C14" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="D14" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="E14" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="F14" t="s">
         <v>13</v>
       </c>
       <c r="G14" t="s">
+        <v>105</v>
+      </c>
+      <c r="H14" t="s">
+        <v>106</v>
+      </c>
+      <c r="I14" t="s">
+        <v>164</v>
+      </c>
+      <c r="J14" t="s">
+        <v>165</v>
+      </c>
+      <c r="K14" t="s">
+        <v>181</v>
+      </c>
+      <c r="L14" t="s">
         <v>110</v>
       </c>
-      <c r="H14" t="s">
-        <v>111</v>
-      </c>
-      <c r="I14" t="s">
-        <v>169</v>
-      </c>
-      <c r="J14" t="s">
-        <v>170</v>
-      </c>
-      <c r="K14" t="s">
-        <v>186</v>
-      </c>
-      <c r="L14" t="s">
-        <v>115</v>
-      </c>
       <c r="M14" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="B15" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="C15" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="D15" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="E15" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="F15" t="s">
         <v>13</v>
       </c>
       <c r="G15" t="s">
+        <v>113</v>
+      </c>
+      <c r="H15" t="s">
+        <v>114</v>
+      </c>
+      <c r="I15" t="s">
+        <v>122</v>
+      </c>
+      <c r="J15" t="s">
+        <v>123</v>
+      </c>
+      <c r="K15" t="s">
+        <v>184</v>
+      </c>
+      <c r="L15" t="s">
         <v>118</v>
       </c>
-      <c r="H15" t="s">
-        <v>119</v>
-      </c>
-      <c r="I15" t="s">
-        <v>127</v>
-      </c>
-      <c r="J15" t="s">
-        <v>128</v>
-      </c>
-      <c r="K15" t="s">
-        <v>189</v>
-      </c>
-      <c r="L15" t="s">
-        <v>123</v>
-      </c>
       <c r="M15" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="B16" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="C16" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="D16" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="E16" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="F16" t="s">
         <v>13</v>
       </c>
       <c r="G16" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
       <c r="H16" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="I16" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="J16" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
       <c r="K16" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="L16" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="M16" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
       <c r="B17" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="C17" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="D17" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="E17" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="F17" t="s">
         <v>13</v>
       </c>
       <c r="G17" t="s">
+        <v>113</v>
+      </c>
+      <c r="H17" t="s">
+        <v>114</v>
+      </c>
+      <c r="I17" t="s">
+        <v>115</v>
+      </c>
+      <c r="J17" t="s">
+        <v>116</v>
+      </c>
+      <c r="K17" t="s">
+        <v>195</v>
+      </c>
+      <c r="L17" t="s">
         <v>118</v>
       </c>
-      <c r="H17" t="s">
-        <v>119</v>
-      </c>
-      <c r="I17" t="s">
-        <v>120</v>
-      </c>
-      <c r="J17" t="s">
-        <v>121</v>
-      </c>
-      <c r="K17" t="s">
-        <v>200</v>
-      </c>
-      <c r="L17" t="s">
-        <v>123</v>
-      </c>
       <c r="M17" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
       <c r="B18" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="C18" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="D18" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="E18" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="F18" t="s">
         <v>13</v>
       </c>
       <c r="G18" t="s">
+        <v>113</v>
+      </c>
+      <c r="H18" t="s">
+        <v>114</v>
+      </c>
+      <c r="I18" t="s">
+        <v>122</v>
+      </c>
+      <c r="J18" t="s">
+        <v>123</v>
+      </c>
+      <c r="K18" t="s">
+        <v>199</v>
+      </c>
+      <c r="L18" t="s">
         <v>118</v>
       </c>
-      <c r="H18" t="s">
-        <v>119</v>
-      </c>
-      <c r="I18" t="s">
-        <v>127</v>
-      </c>
-      <c r="J18" t="s">
-        <v>128</v>
-      </c>
-      <c r="K18" t="s">
-        <v>204</v>
-      </c>
-      <c r="L18" t="s">
-        <v>123</v>
-      </c>
       <c r="M18" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
       <c r="B19" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="C19" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="D19" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="E19" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
       <c r="F19" t="s">
         <v>13</v>
       </c>
       <c r="G19" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="H19" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="I19" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="J19" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="K19" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="L19" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="M19" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="N19" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="O19" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="B20" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="C20" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="D20" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="E20" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="F20" t="s">
         <v>13</v>
       </c>
       <c r="G20" t="s">
+        <v>209</v>
+      </c>
+      <c r="H20" t="s">
+        <v>210</v>
+      </c>
+      <c r="I20" t="s">
+        <v>164</v>
+      </c>
+      <c r="J20" t="s">
+        <v>211</v>
+      </c>
+      <c r="K20" t="s">
+        <v>212</v>
+      </c>
+      <c r="L20" t="s">
+        <v>213</v>
+      </c>
+      <c r="M20" t="s">
         <v>214</v>
       </c>
-      <c r="H20" t="s">
+      <c r="N20" t="s">
         <v>215</v>
       </c>
-      <c r="I20" t="s">
-        <v>169</v>
-      </c>
-      <c r="J20" t="s">
-        <v>216</v>
-      </c>
-      <c r="K20" t="s">
-        <v>217</v>
-      </c>
-      <c r="L20" t="s">
-        <v>218</v>
-      </c>
-      <c r="M20" t="s">
-        <v>219</v>
-      </c>
-      <c r="N20" t="s">
-        <v>220</v>
-      </c>
       <c r="O20" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
     </row>
     <row r="21" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="B21" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="C21" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="D21" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="E21" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="F21" t="s">
         <v>13</v>
       </c>
       <c r="G21" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="H21" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="I21" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="J21" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="K21" t="s">
-        <v>223</v>
+        <v>218</v>
       </c>
       <c r="L21" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="M21" t="s">
-        <v>225</v>
+        <v>220</v>
       </c>
       <c r="P21" t="s">
-        <v>226</v>
+        <v>221</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
       <c r="B22" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="C22" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="D22" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="E22" t="s">
-        <v>228</v>
+        <v>223</v>
       </c>
       <c r="F22" t="s">
         <v>13</v>
       </c>
       <c r="G22" t="s">
+        <v>113</v>
+      </c>
+      <c r="H22" t="s">
+        <v>114</v>
+      </c>
+      <c r="I22" t="s">
+        <v>115</v>
+      </c>
+      <c r="J22" t="s">
+        <v>116</v>
+      </c>
+      <c r="K22" t="s">
+        <v>224</v>
+      </c>
+      <c r="L22" t="s">
         <v>118</v>
       </c>
-      <c r="H22" t="s">
-        <v>119</v>
-      </c>
-      <c r="I22" t="s">
-        <v>120</v>
-      </c>
-      <c r="J22" t="s">
-        <v>121</v>
-      </c>
-      <c r="K22" t="s">
-        <v>229</v>
-      </c>
-      <c r="L22" t="s">
-        <v>123</v>
-      </c>
       <c r="M22" t="s">
-        <v>230</v>
+        <v>225</v>
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>231</v>
+        <v>226</v>
       </c>
       <c r="B23" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="C23" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="D23" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="E23" t="s">
-        <v>232</v>
+        <v>227</v>
       </c>
       <c r="F23" t="s">
         <v>13</v>
       </c>
       <c r="G23" t="s">
+        <v>113</v>
+      </c>
+      <c r="H23" t="s">
+        <v>114</v>
+      </c>
+      <c r="I23" t="s">
+        <v>122</v>
+      </c>
+      <c r="J23" t="s">
+        <v>123</v>
+      </c>
+      <c r="K23" t="s">
+        <v>228</v>
+      </c>
+      <c r="L23" t="s">
         <v>118</v>
       </c>
-      <c r="H23" t="s">
-        <v>119</v>
-      </c>
-      <c r="I23" t="s">
-        <v>127</v>
-      </c>
-      <c r="J23" t="s">
-        <v>128</v>
-      </c>
-      <c r="K23" t="s">
-        <v>233</v>
-      </c>
-      <c r="L23" t="s">
-        <v>123</v>
-      </c>
       <c r="M23" t="s">
-        <v>234</v>
+        <v>229</v>
       </c>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>235</v>
+        <v>230</v>
       </c>
       <c r="B24" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="C24" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="D24" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="E24" t="s">
-        <v>236</v>
+        <v>231</v>
       </c>
       <c r="F24" t="s">
         <v>13</v>
       </c>
       <c r="G24" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="H24" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="I24" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="J24" t="s">
-        <v>237</v>
+        <v>232</v>
       </c>
       <c r="K24" t="s">
-        <v>238</v>
+        <v>233</v>
       </c>
       <c r="L24" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="M24" t="s">
-        <v>237</v>
+        <v>232</v>
       </c>
       <c r="N24" t="s">
-        <v>239</v>
+        <v>234</v>
       </c>
       <c r="O24" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>241</v>
+        <v>236</v>
       </c>
       <c r="B25" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="C25" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="D25" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="E25" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="F25" t="s">
         <v>13</v>
       </c>
       <c r="G25" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="H25" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="I25" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="J25" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="K25" t="s">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="L25" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="M25" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="N25" t="s">
-        <v>245</v>
+        <v>240</v>
       </c>
       <c r="O25" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
       <c r="B26" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="C26" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="D26" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="E26" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
       <c r="F26" t="s">
         <v>13</v>
       </c>
       <c r="G26" t="s">
+        <v>113</v>
+      </c>
+      <c r="H26" t="s">
+        <v>114</v>
+      </c>
+      <c r="I26" t="s">
+        <v>122</v>
+      </c>
+      <c r="J26" t="s">
+        <v>123</v>
+      </c>
+      <c r="K26" t="s">
+        <v>243</v>
+      </c>
+      <c r="L26" t="s">
         <v>118</v>
       </c>
-      <c r="H26" t="s">
-        <v>119</v>
-      </c>
-      <c r="I26" t="s">
-        <v>127</v>
-      </c>
-      <c r="J26" t="s">
-        <v>128</v>
-      </c>
-      <c r="K26" t="s">
-        <v>248</v>
-      </c>
-      <c r="L26" t="s">
-        <v>123</v>
-      </c>
       <c r="M26" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="B27" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="C27" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="D27" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="E27" t="s">
-        <v>251</v>
+        <v>246</v>
       </c>
       <c r="F27" t="s">
         <v>13</v>
       </c>
       <c r="G27" t="s">
+        <v>113</v>
+      </c>
+      <c r="H27" t="s">
+        <v>114</v>
+      </c>
+      <c r="I27" t="s">
+        <v>122</v>
+      </c>
+      <c r="J27" t="s">
+        <v>123</v>
+      </c>
+      <c r="K27" t="s">
+        <v>247</v>
+      </c>
+      <c r="L27" t="s">
         <v>118</v>
       </c>
-      <c r="H27" t="s">
-        <v>119</v>
-      </c>
-      <c r="I27" t="s">
-        <v>127</v>
-      </c>
-      <c r="J27" t="s">
-        <v>128</v>
-      </c>
-      <c r="K27" t="s">
-        <v>252</v>
-      </c>
-      <c r="L27" t="s">
-        <v>123</v>
-      </c>
       <c r="M27" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="B28" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="C28" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="D28" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="E28" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="F28" t="s">
         <v>13</v>
       </c>
       <c r="G28" t="s">
+        <v>113</v>
+      </c>
+      <c r="H28" t="s">
+        <v>114</v>
+      </c>
+      <c r="I28" t="s">
+        <v>115</v>
+      </c>
+      <c r="J28" t="s">
+        <v>116</v>
+      </c>
+      <c r="K28" t="s">
+        <v>251</v>
+      </c>
+      <c r="L28" t="s">
         <v>118</v>
       </c>
-      <c r="H28" t="s">
-        <v>119</v>
-      </c>
-      <c r="I28" t="s">
-        <v>120</v>
-      </c>
-      <c r="J28" t="s">
-        <v>121</v>
-      </c>
-      <c r="K28" t="s">
-        <v>256</v>
-      </c>
-      <c r="L28" t="s">
-        <v>123</v>
-      </c>
       <c r="M28" t="s">
-        <v>257</v>
+        <v>252</v>
       </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
       <c r="B29" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="C29" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="D29" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="E29" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="F29" t="s">
         <v>13</v>
       </c>
       <c r="G29" t="s">
+        <v>113</v>
+      </c>
+      <c r="H29" t="s">
+        <v>114</v>
+      </c>
+      <c r="I29" t="s">
+        <v>122</v>
+      </c>
+      <c r="J29" t="s">
+        <v>123</v>
+      </c>
+      <c r="K29" t="s">
+        <v>255</v>
+      </c>
+      <c r="L29" t="s">
         <v>118</v>
       </c>
-      <c r="H29" t="s">
-        <v>119</v>
-      </c>
-      <c r="I29" t="s">
-        <v>127</v>
-      </c>
-      <c r="J29" t="s">
-        <v>128</v>
-      </c>
-      <c r="K29" t="s">
-        <v>260</v>
-      </c>
-      <c r="L29" t="s">
-        <v>123</v>
-      </c>
       <c r="M29" t="s">
-        <v>261</v>
+        <v>256</v>
       </c>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="B30" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="C30" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="D30" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="E30" t="s">
-        <v>263</v>
+        <v>258</v>
       </c>
       <c r="F30" t="s">
         <v>13</v>
       </c>
       <c r="G30" t="s">
+        <v>113</v>
+      </c>
+      <c r="H30" t="s">
+        <v>114</v>
+      </c>
+      <c r="I30" t="s">
+        <v>122</v>
+      </c>
+      <c r="J30" t="s">
+        <v>123</v>
+      </c>
+      <c r="K30" t="s">
+        <v>259</v>
+      </c>
+      <c r="L30" t="s">
         <v>118</v>
       </c>
-      <c r="H30" t="s">
-        <v>119</v>
-      </c>
-      <c r="I30" t="s">
-        <v>127</v>
-      </c>
-      <c r="J30" t="s">
-        <v>128</v>
-      </c>
-      <c r="K30" t="s">
-        <v>264</v>
-      </c>
-      <c r="L30" t="s">
-        <v>123</v>
-      </c>
       <c r="M30" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
     </row>
     <row r="31" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>266</v>
+        <v>261</v>
       </c>
       <c r="B31" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="C31" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="D31" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="E31" t="s">
-        <v>267</v>
+        <v>262</v>
       </c>
       <c r="F31" t="s">
         <v>13</v>
       </c>
       <c r="G31" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="H31" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="I31" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="J31" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="K31" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
       <c r="L31" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="M31" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="P31" t="s">
-        <v>226</v>
+        <v>221</v>
       </c>
     </row>
     <row r="32" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="B32" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="C32" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="D32" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="E32" t="s">
-        <v>271</v>
+        <v>266</v>
       </c>
       <c r="F32" t="s">
         <v>13</v>
       </c>
       <c r="G32" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="H32" t="s">
-        <v>272</v>
+        <v>267</v>
       </c>
       <c r="I32" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="J32" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="K32" t="s">
-        <v>273</v>
+        <v>268</v>
       </c>
       <c r="M32" t="s">
-        <v>274</v>
+        <v>269</v>
       </c>
       <c r="Q32" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="R32" t="s">
-        <v>276</v>
+        <v>271</v>
       </c>
     </row>
     <row r="33" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
+        <v>272</v>
+      </c>
+      <c r="B33" t="s">
+        <v>102</v>
+      </c>
+      <c r="C33" t="s">
+        <v>265</v>
+      </c>
+      <c r="D33" t="s">
+        <v>89</v>
+      </c>
+      <c r="E33" t="s">
+        <v>273</v>
+      </c>
+      <c r="F33" t="s">
+        <v>274</v>
+      </c>
+      <c r="G33" t="s">
+        <v>105</v>
+      </c>
+      <c r="H33" t="s">
+        <v>275</v>
+      </c>
+      <c r="I33" t="s">
+        <v>107</v>
+      </c>
+      <c r="J33" t="s">
+        <v>272</v>
+      </c>
+      <c r="L33" t="s">
+        <v>276</v>
+      </c>
+      <c r="M33" t="s">
+        <v>272</v>
+      </c>
+      <c r="Q33" t="s">
         <v>277</v>
       </c>
-      <c r="B33" t="s">
-        <v>107</v>
-      </c>
-      <c r="C33" t="s">
-        <v>270</v>
-      </c>
-      <c r="D33" t="s">
-        <v>95</v>
-      </c>
-      <c r="E33" t="s">
-        <v>278</v>
-      </c>
-      <c r="F33" t="s">
-        <v>279</v>
-      </c>
-      <c r="G33" t="s">
-        <v>110</v>
-      </c>
-      <c r="H33" t="s">
-        <v>280</v>
-      </c>
-      <c r="I33" t="s">
-        <v>112</v>
-      </c>
-      <c r="J33" t="s">
-        <v>277</v>
-      </c>
-      <c r="L33" t="s">
-        <v>281</v>
-      </c>
-      <c r="M33" t="s">
-        <v>277</v>
-      </c>
-      <c r="Q33" t="s">
-        <v>282</v>
-      </c>
       <c r="R33" t="s">
-        <v>276</v>
+        <v>271</v>
       </c>
     </row>
     <row r="34" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
+        <v>278</v>
+      </c>
+      <c r="B34" t="s">
+        <v>102</v>
+      </c>
+      <c r="C34" t="s">
+        <v>265</v>
+      </c>
+      <c r="D34" t="s">
+        <v>89</v>
+      </c>
+      <c r="E34" t="s">
+        <v>279</v>
+      </c>
+      <c r="G34" t="s">
+        <v>280</v>
+      </c>
+      <c r="H34" t="s">
+        <v>281</v>
+      </c>
+      <c r="I34" t="s">
+        <v>107</v>
+      </c>
+      <c r="J34" t="s">
+        <v>278</v>
+      </c>
+      <c r="K34" t="s">
+        <v>282</v>
+      </c>
+      <c r="L34" t="s">
         <v>283</v>
       </c>
-      <c r="B34" t="s">
-        <v>107</v>
-      </c>
-      <c r="C34" t="s">
-        <v>270</v>
-      </c>
-      <c r="D34" t="s">
-        <v>95</v>
-      </c>
-      <c r="E34" t="s">
+      <c r="M34" t="s">
         <v>284</v>
       </c>
-      <c r="G34" t="s">
+      <c r="Q34" t="s">
         <v>285</v>
       </c>
-      <c r="H34" t="s">
-        <v>286</v>
-      </c>
-      <c r="I34" t="s">
-        <v>112</v>
-      </c>
-      <c r="J34" t="s">
-        <v>283</v>
-      </c>
-      <c r="K34" t="s">
-        <v>287</v>
-      </c>
-      <c r="L34" t="s">
-        <v>288</v>
-      </c>
-      <c r="M34" t="s">
-        <v>289</v>
-      </c>
-      <c r="Q34" t="s">
-        <v>290</v>
-      </c>
       <c r="R34" t="s">
-        <v>276</v>
+        <v>271</v>
       </c>
     </row>
     <row r="35" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>291</v>
+        <v>286</v>
       </c>
       <c r="B35" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="C35" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="D35" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="E35" t="s">
-        <v>292</v>
+        <v>287</v>
       </c>
       <c r="F35" t="s">
         <v>13</v>
       </c>
       <c r="G35" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
       <c r="H35" t="s">
+        <v>281</v>
+      </c>
+      <c r="I35" t="s">
+        <v>107</v>
+      </c>
+      <c r="J35" t="s">
         <v>286</v>
       </c>
-      <c r="I35" t="s">
-        <v>112</v>
-      </c>
-      <c r="J35" t="s">
-        <v>291</v>
-      </c>
       <c r="K35" t="s">
-        <v>293</v>
+        <v>288</v>
       </c>
       <c r="L35" t="s">
-        <v>288</v>
+        <v>283</v>
       </c>
       <c r="M35" t="s">
-        <v>294</v>
+        <v>289</v>
       </c>
       <c r="Q35" t="s">
-        <v>295</v>
+        <v>290</v>
       </c>
       <c r="R35" t="s">
-        <v>276</v>
+        <v>271</v>
       </c>
     </row>
   </sheetData>
@@ -3468,82 +3405,46 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>296</v>
+        <v>291</v>
       </c>
       <c r="B2" t="s">
-        <v>297</v>
+        <v>292</v>
       </c>
       <c r="C2" t="s">
-        <v>298</v>
+        <v>293</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>299</v>
+        <v>294</v>
       </c>
       <c r="B3" t="s">
-        <v>300</v>
+        <v>295</v>
       </c>
       <c r="C3" t="s">
-        <v>298</v>
+        <v>293</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>301</v>
+        <v>296</v>
       </c>
       <c r="B4" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
       <c r="C4" t="s">
-        <v>298</v>
+        <v>293</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>302</v>
+        <v>297</v>
       </c>
       <c r="B5" t="s">
-        <v>303</v>
+        <v>298</v>
       </c>
       <c r="C5" t="s">
-        <v>298</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
-  <cols>
-    <col min="1" max="3" width="20" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>304</v>
-      </c>
-      <c r="B2" t="s">
-        <v>305</v>
-      </c>
-      <c r="C2" t="s">
-        <v>306</v>
+        <v>293</v>
       </c>
     </row>
   </sheetData>

</xml_diff>